<commit_message>
vault backup: 2026-08-21 11:56:42
</commit_message>
<xml_diff>
--- a/ContabilidadeFinanceira/Aulas/08.20/T4_Loja Sedução_Planilha.xlsx
+++ b/ContabilidadeFinanceira/Aulas/08.20/T4_Loja Sedução_Planilha.xlsx
@@ -37,15 +37,27 @@
         </r>
       </text>
     </comment>
-    <comment ref="D25" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Empréstimo 1% a.m., 5 parcelas anuais</t>
+    <comment ref="D24" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Parcela do ano 1: vence ~11 meses após a data do balanço, dentro de 12m -&gt; circulante</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D26" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Parcelas dos anos 2-5</t>
         </r>
       </text>
     </comment>
@@ -85,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E53" authorId="0">
+    <comment ref="E54" authorId="0">
       <text>
         <r>
           <rPr>
@@ -145,7 +157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H29" authorId="0">
+    <comment ref="H30" authorId="0">
       <text>
         <r>
           <rPr>
@@ -157,7 +169,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H35" authorId="0">
+    <comment ref="H36" authorId="0">
       <text>
         <r>
           <rPr>
@@ -169,7 +181,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H51" authorId="0">
+    <comment ref="H52" authorId="0">
       <text>
         <r>
           <rPr>
@@ -193,7 +205,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I29" authorId="0">
+    <comment ref="I30" authorId="0">
       <text>
         <r>
           <rPr>
@@ -241,7 +253,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J29" authorId="0">
+    <comment ref="J30" authorId="0">
       <text>
         <r>
           <rPr>
@@ -253,7 +265,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J40" authorId="0">
+    <comment ref="J41" authorId="0">
       <text>
         <r>
           <rPr>
@@ -277,7 +289,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K45" authorId="0">
+    <comment ref="K46" authorId="0">
       <text>
         <r>
           <rPr>
@@ -301,7 +313,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M62" authorId="0">
+    <comment ref="M63" authorId="0">
       <text>
         <r>
           <rPr>
@@ -313,7 +325,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M63" authorId="0">
+    <comment ref="M64" authorId="0">
       <text>
         <r>
           <rPr>
@@ -337,7 +349,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N60" authorId="0">
+    <comment ref="N61" authorId="0">
       <text>
         <r>
           <rPr>
@@ -397,7 +409,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P29" authorId="0">
+    <comment ref="P30" authorId="0">
       <text>
         <r>
           <rPr>
@@ -409,7 +421,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P35" authorId="0">
+    <comment ref="P36" authorId="0">
       <text>
         <r>
           <rPr>
@@ -445,7 +457,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S39" authorId="0">
+    <comment ref="S40" authorId="0">
       <text>
         <r>
           <rPr>
@@ -465,11 +477,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Quita empréstimo 50.000 + juros acumulados 1.000 (jul+ago)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T29" authorId="0">
+          <t xml:space="preserve">Quita empréstimo 50.000 (CP+LP) + juros acumulados 1.000</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T30" authorId="0">
       <text>
         <r>
           <rPr>
@@ -481,7 +493,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T54" authorId="0">
+    <comment ref="T55" authorId="0">
       <text>
         <r>
           <rPr>
@@ -517,7 +529,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U29" authorId="0">
+    <comment ref="U30" authorId="0">
       <text>
         <r>
           <rPr>
@@ -529,7 +541,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U45" authorId="0">
+    <comment ref="U46" authorId="0">
       <text>
         <r>
           <rPr>
@@ -541,7 +553,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U54" authorId="0">
+    <comment ref="U55" authorId="0">
       <text>
         <r>
           <rPr>
@@ -553,7 +565,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V63" authorId="0">
+    <comment ref="V64" authorId="0">
       <text>
         <r>
           <rPr>
@@ -570,7 +582,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
   <si>
     <t xml:space="preserve">Transações, por Número</t>
   </si>
@@ -639,6 +651,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Juros a Pagar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Empréstimos e Financiamentos (CP)</t>
   </si>
   <si>
     <t xml:space="preserve">Passivo Não Circulante</t>
@@ -1506,7 +1521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AU63"/>
+  <dimension ref="A1:AU64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.09"/>
@@ -2395,7 +2410,7 @@
       <c r="I20" s="14"/>
       <c r="J20" s="14"/>
       <c r="K20" s="19" t="n">
-        <f aca="false">0.3*M44</f>
+        <f aca="false">0.3*M45</f>
         <v>15435</v>
       </c>
       <c r="L20" s="14"/>
@@ -2411,7 +2426,7 @@
       <c r="S20" s="14"/>
       <c r="T20" s="14"/>
       <c r="U20" s="19" t="n">
-        <f aca="false">-M20-U45</f>
+        <f aca="false">-M20-U46</f>
         <v>-2460</v>
       </c>
       <c r="V20" s="18" t="n">
@@ -2475,7 +2490,7 @@
         <v>21</v>
       </c>
       <c r="L22" s="24" t="n">
-        <f aca="false">0.4*M46</f>
+        <f aca="false">0.4*M47</f>
         <v>14406</v>
       </c>
       <c r="M22" s="24" t="n">
@@ -2511,45 +2526,30 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
-      <c r="R24" s="14"/>
-      <c r="S24" s="14"/>
-      <c r="T24" s="14"/>
-      <c r="U24" s="14"/>
-      <c r="V24" s="13"/>
-      <c r="W24" s="14"/>
-      <c r="X24" s="14"/>
-      <c r="Y24" s="14"/>
-      <c r="Z24" s="14"/>
-      <c r="AA24" s="14"/>
-      <c r="AB24" s="14"/>
-      <c r="AC24" s="14"/>
+      <c r="D24" s="16" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M24" s="24" t="n">
+        <f aca="false">SUM(B24:L24)</f>
+        <v>10000</v>
+      </c>
+      <c r="T24" s="16" t="n">
+        <v>-10000</v>
+      </c>
+      <c r="V24" s="24" t="n">
+        <f aca="false">SUM(M24:U24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="12" t="s">
         <v>24</v>
       </c>
       <c r="B25" s="13"/>
-      <c r="D25" s="17" t="n">
-        <v>50000</v>
-      </c>
+      <c r="D25" s="14"/>
       <c r="E25" s="14"/>
       <c r="F25" s="14"/>
       <c r="G25" s="14"/>
@@ -2558,24 +2558,16 @@
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
       <c r="L25" s="14"/>
-      <c r="M25" s="18" t="n">
-        <f aca="false">SUM(B25:L25)</f>
-        <v>50000</v>
-      </c>
+      <c r="M25" s="13"/>
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
       <c r="P25" s="14"/>
       <c r="Q25" s="14"/>
       <c r="R25" s="14"/>
       <c r="S25" s="14"/>
-      <c r="T25" s="17" t="n">
-        <v>-50000</v>
-      </c>
+      <c r="T25" s="14"/>
       <c r="U25" s="14"/>
-      <c r="V25" s="18" t="n">
-        <f aca="false">SUM(M25:U25)</f>
-        <v>0</v>
-      </c>
+      <c r="V25" s="13"/>
       <c r="W25" s="14"/>
       <c r="X25" s="14"/>
       <c r="Y25" s="14"/>
@@ -2589,7 +2581,9 @@
         <v>25</v>
       </c>
       <c r="B26" s="13"/>
-      <c r="D26" s="14"/>
+      <c r="D26" s="17" t="n">
+        <v>40000</v>
+      </c>
       <c r="E26" s="14"/>
       <c r="F26" s="14"/>
       <c r="G26" s="14"/>
@@ -2600,7 +2594,7 @@
       <c r="L26" s="14"/>
       <c r="M26" s="18" t="n">
         <f aca="false">SUM(B26:L26)</f>
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="N26" s="14"/>
       <c r="O26" s="14"/>
@@ -2608,7 +2602,9 @@
       <c r="Q26" s="14"/>
       <c r="R26" s="14"/>
       <c r="S26" s="14"/>
-      <c r="T26" s="14"/>
+      <c r="T26" s="17" t="n">
+        <v>-40000</v>
+      </c>
       <c r="U26" s="14"/>
       <c r="V26" s="18" t="n">
         <f aca="false">SUM(M26:U26)</f>
@@ -2623,7 +2619,7 @@
       <c r="AC26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="15" t="s">
         <v>26</v>
       </c>
       <c r="B27" s="13"/>
@@ -2636,7 +2632,10 @@
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
       <c r="L27" s="14"/>
-      <c r="M27" s="13"/>
+      <c r="M27" s="18" t="n">
+        <f aca="false">SUM(B27:L27)</f>
+        <v>0</v>
+      </c>
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
       <c r="P27" s="14"/>
@@ -2645,7 +2644,10 @@
       <c r="S27" s="14"/>
       <c r="T27" s="14"/>
       <c r="U27" s="14"/>
-      <c r="V27" s="13"/>
+      <c r="V27" s="18" t="n">
+        <f aca="false">SUM(M27:U27)</f>
+        <v>0</v>
+      </c>
       <c r="W27" s="14"/>
       <c r="X27" s="14"/>
       <c r="Y27" s="14"/>
@@ -2655,13 +2657,10 @@
       <c r="AC27" s="14"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="12" t="s">
         <v>27</v>
       </c>
       <c r="B28" s="13"/>
-      <c r="C28" s="16" t="n">
-        <v>80000</v>
-      </c>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
@@ -2671,10 +2670,7 @@
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
       <c r="L28" s="14"/>
-      <c r="M28" s="18" t="n">
-        <f aca="false">SUM(B28:L28)</f>
-        <v>80000</v>
-      </c>
+      <c r="M28" s="13"/>
       <c r="N28" s="14"/>
       <c r="O28" s="14"/>
       <c r="P28" s="14"/>
@@ -2683,10 +2679,7 @@
       <c r="S28" s="14"/>
       <c r="T28" s="14"/>
       <c r="U28" s="14"/>
-      <c r="V28" s="18" t="n">
-        <f aca="false">SUM(M28:U28)</f>
-        <v>80000</v>
-      </c>
+      <c r="V28" s="13"/>
       <c r="W28" s="14"/>
       <c r="X28" s="14"/>
       <c r="Y28" s="14"/>
@@ -2700,53 +2693,33 @@
         <v>28</v>
       </c>
       <c r="B29" s="13"/>
+      <c r="C29" s="16" t="n">
+        <v>80000</v>
+      </c>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
       <c r="F29" s="14"/>
       <c r="G29" s="14"/>
-      <c r="H29" s="17" t="n">
-        <v>56000</v>
-      </c>
-      <c r="I29" s="17" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="J29" s="17" t="n">
-        <v>-2550</v>
-      </c>
-      <c r="K29" s="19" t="n">
-        <f aca="false">-0.3*M44</f>
-        <v>-15435</v>
-      </c>
-      <c r="L29" s="19" t="n">
-        <f aca="false">-0.4*M46</f>
-        <v>-14406</v>
-      </c>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="14"/>
       <c r="M29" s="18" t="n">
         <f aca="false">SUM(B29:L29)</f>
-        <v>21609</v>
+        <v>80000</v>
       </c>
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
-      <c r="P29" s="17" t="n">
-        <v>49000</v>
-      </c>
+      <c r="P29" s="14"/>
       <c r="Q29" s="14"/>
-      <c r="R29" s="17" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="S29" s="17" t="n">
-        <v>-1200</v>
-      </c>
-      <c r="T29" s="17" t="n">
-        <v>-500</v>
-      </c>
-      <c r="U29" s="19" t="n">
-        <f aca="false">-1500-550+U45</f>
-        <v>-15025</v>
-      </c>
+      <c r="R29" s="14"/>
+      <c r="S29" s="14"/>
+      <c r="T29" s="14"/>
+      <c r="U29" s="14"/>
       <c r="V29" s="18" t="n">
         <f aca="false">SUM(M29:U29)</f>
-        <v>51884</v>
+        <v>80000</v>
       </c>
       <c r="W29" s="14"/>
       <c r="X29" s="14"/>
@@ -2757,92 +2730,57 @@
       <c r="AC29" s="14"/>
     </row>
     <row r="30" s="25" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="21" t="n">
-        <f aca="false">SUM(B18:B29)</f>
-        <v>0</v>
-      </c>
-      <c r="C30" s="22" t="n">
-        <f aca="false">SUM(C18:C29)</f>
-        <v>80000</v>
-      </c>
-      <c r="D30" s="21" t="n">
-        <f aca="false">SUM(D18:D29)</f>
-        <v>50000</v>
-      </c>
-      <c r="E30" s="21" t="n">
-        <f aca="false">SUM(E18:E29)</f>
-        <v>0</v>
-      </c>
-      <c r="F30" s="21" t="n">
-        <f aca="false">SUM(F18:F29)</f>
-        <v>0</v>
-      </c>
-      <c r="G30" s="21" t="n">
-        <f aca="false">SUM(G18:G29)</f>
-        <v>0</v>
-      </c>
-      <c r="H30" s="21" t="n">
-        <f aca="false">SUM(H18:H29)</f>
-        <v>76000</v>
-      </c>
-      <c r="I30" s="21" t="n">
-        <f aca="false">SUM(I18:I29)</f>
-        <v>-1000</v>
-      </c>
-      <c r="J30" s="21" t="n">
-        <f aca="false">SUM(J18:J29)</f>
-        <v>-2050</v>
-      </c>
-      <c r="K30" s="21" t="n">
-        <f aca="false">SUM(K18:K29)</f>
-        <v>0</v>
-      </c>
-      <c r="L30" s="21" t="n">
-        <f aca="false">SUM(L18:L29)</f>
-        <v>0</v>
-      </c>
-      <c r="M30" s="21" t="n">
-        <f aca="false">SUM(M18:M29)</f>
-        <v>202950</v>
-      </c>
-      <c r="N30" s="21" t="n">
-        <f aca="false">SUM(N18:N29)</f>
-        <v>-15406</v>
-      </c>
-      <c r="O30" s="21" t="n">
-        <f aca="false">SUM(O18:O29)</f>
-        <v>15000</v>
-      </c>
-      <c r="P30" s="21" t="n">
-        <f aca="false">SUM(P18:P29)</f>
-        <v>29000</v>
-      </c>
-      <c r="Q30" s="21" t="n">
-        <f aca="false">SUM(Q18:Q29)</f>
-        <v>250</v>
-      </c>
-      <c r="R30" s="21" t="n">
-        <f aca="false">SUM(R18:R29)</f>
-        <v>-1000</v>
-      </c>
-      <c r="S30" s="21" t="n">
-        <f aca="false">SUM(S18:S29)</f>
+      <c r="B30" s="13"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="17" t="n">
+        <v>56000</v>
+      </c>
+      <c r="I30" s="17" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="J30" s="17" t="n">
+        <v>-2550</v>
+      </c>
+      <c r="K30" s="19" t="n">
+        <f aca="false">-0.3*M45</f>
+        <v>-15435</v>
+      </c>
+      <c r="L30" s="19" t="n">
+        <f aca="false">-0.4*M47</f>
+        <v>-14406</v>
+      </c>
+      <c r="M30" s="18" t="n">
+        <f aca="false">SUM(B30:L30)</f>
+        <v>21609</v>
+      </c>
+      <c r="N30" s="14"/>
+      <c r="O30" s="14"/>
+      <c r="P30" s="17" t="n">
+        <v>49000</v>
+      </c>
+      <c r="Q30" s="14"/>
+      <c r="R30" s="17" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="S30" s="17" t="n">
         <v>-1200</v>
       </c>
-      <c r="T30" s="21" t="n">
-        <f aca="false">SUM(T18:T29)</f>
-        <v>-51000</v>
-      </c>
-      <c r="U30" s="21" t="n">
-        <f aca="false">SUM(U18:U29)</f>
-        <v>-17485</v>
-      </c>
-      <c r="V30" s="21" t="n">
-        <f aca="false">SUM(V18:V29)</f>
-        <v>161109</v>
+      <c r="T30" s="17" t="n">
+        <v>-500</v>
+      </c>
+      <c r="U30" s="19" t="n">
+        <f aca="false">-1500-550+U46</f>
+        <v>-15025</v>
+      </c>
+      <c r="V30" s="18" t="n">
+        <f aca="false">SUM(M30:U30)</f>
+        <v>51884</v>
       </c>
       <c r="W30" s="14"/>
       <c r="X30" s="14"/>
@@ -2853,26 +2791,93 @@
       <c r="AC30" s="14"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
-      <c r="O31" s="14"/>
-      <c r="P31" s="14"/>
-      <c r="Q31" s="14"/>
-      <c r="R31" s="14"/>
-      <c r="S31" s="14"/>
-      <c r="T31" s="14"/>
-      <c r="U31" s="14"/>
-      <c r="V31" s="14"/>
+      <c r="A31" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <f aca="false">SUM(B18:B30)</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="22" t="n">
+        <f aca="false">SUM(C18:C30)</f>
+        <v>80000</v>
+      </c>
+      <c r="D31" s="21" t="n">
+        <f aca="false">SUM(D18:D30)</f>
+        <v>50000</v>
+      </c>
+      <c r="E31" s="21" t="n">
+        <f aca="false">SUM(E18:E30)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="21" t="n">
+        <f aca="false">SUM(F18:F30)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="21" t="n">
+        <f aca="false">SUM(G18:G30)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="21" t="n">
+        <f aca="false">SUM(H18:H30)</f>
+        <v>76000</v>
+      </c>
+      <c r="I31" s="21" t="n">
+        <f aca="false">SUM(I18:I30)</f>
+        <v>-1000</v>
+      </c>
+      <c r="J31" s="21" t="n">
+        <f aca="false">SUM(J18:J30)</f>
+        <v>-2050</v>
+      </c>
+      <c r="K31" s="21" t="n">
+        <f aca="false">SUM(K18:K30)</f>
+        <v>0</v>
+      </c>
+      <c r="L31" s="21" t="n">
+        <f aca="false">SUM(L18:L30)</f>
+        <v>0</v>
+      </c>
+      <c r="M31" s="21" t="n">
+        <f aca="false">SUM(M18:M30)</f>
+        <v>202950</v>
+      </c>
+      <c r="N31" s="21" t="n">
+        <f aca="false">SUM(N18:N30)</f>
+        <v>-15406</v>
+      </c>
+      <c r="O31" s="21" t="n">
+        <f aca="false">SUM(O18:O30)</f>
+        <v>15000</v>
+      </c>
+      <c r="P31" s="21" t="n">
+        <f aca="false">SUM(P18:P30)</f>
+        <v>29000</v>
+      </c>
+      <c r="Q31" s="21" t="n">
+        <f aca="false">SUM(Q18:Q30)</f>
+        <v>250</v>
+      </c>
+      <c r="R31" s="21" t="n">
+        <f aca="false">SUM(R18:R30)</f>
+        <v>-1000</v>
+      </c>
+      <c r="S31" s="21" t="n">
+        <f aca="false">SUM(S18:S30)</f>
+        <v>-1200</v>
+      </c>
+      <c r="T31" s="21" t="n">
+        <f aca="false">SUM(T18:T30)</f>
+        <v>-51000</v>
+      </c>
+      <c r="U31" s="21" t="n">
+        <f aca="false">SUM(U18:U30)</f>
+        <v>-17485</v>
+      </c>
+      <c r="V31" s="21" t="n">
+        <f aca="false">SUM(V18:V30)</f>
+        <v>161109</v>
+      </c>
       <c r="W31" s="14"/>
       <c r="X31" s="14"/>
       <c r="Y31" s="14"/>
@@ -2882,159 +2887,152 @@
       <c r="AC31" s="14"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="27" t="n">
-        <f aca="false">B15-B30</f>
-        <v>0</v>
-      </c>
-      <c r="C32" s="22" t="n">
-        <f aca="false">C15-C30</f>
-        <v>0</v>
-      </c>
-      <c r="D32" s="27" t="n">
-        <f aca="false">D15-D30</f>
-        <v>0</v>
-      </c>
-      <c r="E32" s="27" t="n">
-        <f aca="false">E15-E30</f>
-        <v>0</v>
-      </c>
-      <c r="F32" s="27" t="n">
-        <f aca="false">F15-F30</f>
-        <v>0</v>
-      </c>
-      <c r="G32" s="27" t="n">
-        <f aca="false">G15-G30</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="27" t="n">
-        <f aca="false">H15-H30</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="27" t="n">
-        <f aca="false">I15-I30</f>
-        <v>0</v>
-      </c>
-      <c r="J32" s="27" t="n">
-        <f aca="false">J15-J30</f>
-        <v>0</v>
-      </c>
-      <c r="K32" s="27" t="n">
-        <f aca="false">K15-K30</f>
-        <v>0</v>
-      </c>
-      <c r="L32" s="27" t="n">
-        <f aca="false">L15-L30</f>
-        <v>0</v>
-      </c>
-      <c r="M32" s="27" t="n">
-        <f aca="false">M15-M30</f>
-        <v>0</v>
-      </c>
-      <c r="N32" s="27" t="n">
-        <f aca="false">N15-N30</f>
-        <v>0</v>
-      </c>
-      <c r="O32" s="27" t="n">
-        <f aca="false">O15-O30</f>
-        <v>0</v>
-      </c>
-      <c r="P32" s="27" t="n">
-        <f aca="false">P15-P30</f>
-        <v>0</v>
-      </c>
-      <c r="Q32" s="27" t="n">
-        <f aca="false">Q15-Q30</f>
-        <v>0</v>
-      </c>
-      <c r="R32" s="27" t="n">
-        <f aca="false">R15-R30</f>
-        <v>0</v>
-      </c>
-      <c r="S32" s="27" t="n">
-        <f aca="false">S15-S30</f>
-        <v>0</v>
-      </c>
-      <c r="T32" s="27" t="n">
-        <f aca="false">T15-T30</f>
-        <v>0</v>
-      </c>
-      <c r="U32" s="27" t="n">
-        <f aca="false">U15-U30</f>
-        <v>0</v>
-      </c>
-      <c r="V32" s="27" t="n">
-        <f aca="false">V15-V30</f>
-        <v>0</v>
-      </c>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
-      <c r="AD32" s="29"/>
+      <c r="B32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
+      <c r="O32" s="14"/>
+      <c r="P32" s="14"/>
+      <c r="Q32" s="14"/>
+      <c r="R32" s="14"/>
+      <c r="S32" s="14"/>
+      <c r="T32" s="14"/>
+      <c r="U32" s="14"/>
+      <c r="V32" s="14"/>
+      <c r="W32" s="14"/>
+      <c r="X32" s="14"/>
+      <c r="Y32" s="14"/>
+      <c r="Z32" s="14"/>
+      <c r="AA32" s="14"/>
+      <c r="AB32" s="14"/>
+      <c r="AC32" s="14"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="14"/>
-      <c r="O33" s="14"/>
-      <c r="P33" s="14"/>
-      <c r="Q33" s="14"/>
-      <c r="R33" s="14"/>
-      <c r="S33" s="14"/>
-      <c r="T33" s="14"/>
-      <c r="U33" s="14"/>
-      <c r="V33" s="14"/>
-      <c r="W33" s="14"/>
-      <c r="X33" s="14"/>
-      <c r="Y33" s="14"/>
-      <c r="Z33" s="14"/>
-      <c r="AA33" s="14"/>
-      <c r="AB33" s="14"/>
-      <c r="AC33" s="14"/>
+      <c r="A33" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="27" t="n">
+        <f aca="false">B15-B31</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="22" t="n">
+        <f aca="false">C15-C31</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="27" t="n">
+        <f aca="false">D15-D31</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="27" t="n">
+        <f aca="false">E15-E31</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="27" t="n">
+        <f aca="false">F15-F31</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="27" t="n">
+        <f aca="false">G15-G31</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="27" t="n">
+        <f aca="false">H15-H31</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <f aca="false">I15-I31</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="27" t="n">
+        <f aca="false">J15-J31</f>
+        <v>0</v>
+      </c>
+      <c r="K33" s="27" t="n">
+        <f aca="false">K15-K31</f>
+        <v>0</v>
+      </c>
+      <c r="L33" s="27" t="n">
+        <f aca="false">L15-L31</f>
+        <v>0</v>
+      </c>
+      <c r="M33" s="27" t="n">
+        <f aca="false">M15-M31</f>
+        <v>0</v>
+      </c>
+      <c r="N33" s="27" t="n">
+        <f aca="false">N15-N31</f>
+        <v>0</v>
+      </c>
+      <c r="O33" s="27" t="n">
+        <f aca="false">O15-O31</f>
+        <v>0</v>
+      </c>
+      <c r="P33" s="27" t="n">
+        <f aca="false">P15-P31</f>
+        <v>0</v>
+      </c>
+      <c r="Q33" s="27" t="n">
+        <f aca="false">Q15-Q31</f>
+        <v>0</v>
+      </c>
+      <c r="R33" s="27" t="n">
+        <f aca="false">R15-R31</f>
+        <v>0</v>
+      </c>
+      <c r="S33" s="27" t="n">
+        <f aca="false">S15-S31</f>
+        <v>0</v>
+      </c>
+      <c r="T33" s="27" t="n">
+        <f aca="false">T15-T31</f>
+        <v>0</v>
+      </c>
+      <c r="U33" s="27" t="n">
+        <f aca="false">U15-U31</f>
+        <v>0</v>
+      </c>
+      <c r="V33" s="27" t="n">
+        <f aca="false">V15-V31</f>
+        <v>0</v>
+      </c>
+      <c r="W33" s="28"/>
+      <c r="X33" s="28"/>
+      <c r="Y33" s="28"/>
+      <c r="Z33" s="28"/>
+      <c r="AA33" s="28"/>
+      <c r="AB33" s="28"/>
+      <c r="AC33" s="28"/>
+      <c r="AD33" s="29"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="B34" s="31"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="N34" s="31"/>
-      <c r="O34" s="31"/>
-      <c r="P34" s="31"/>
-      <c r="Q34" s="31"/>
-      <c r="R34" s="31"/>
-      <c r="S34" s="31"/>
-      <c r="T34" s="31"/>
-      <c r="U34" s="31"/>
-      <c r="V34" s="32" t="s">
-        <v>33</v>
-      </c>
+      <c r="B34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
+      <c r="O34" s="14"/>
+      <c r="P34" s="14"/>
+      <c r="Q34" s="14"/>
+      <c r="R34" s="14"/>
+      <c r="S34" s="14"/>
+      <c r="T34" s="14"/>
+      <c r="U34" s="14"/>
+      <c r="V34" s="14"/>
       <c r="W34" s="14"/>
       <c r="X34" s="14"/>
       <c r="Y34" s="14"/>
@@ -3044,38 +3042,32 @@
       <c r="AC34" s="14"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="31"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="31"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="31"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
+      <c r="J35" s="31"/>
+      <c r="K35" s="31"/>
+      <c r="L35" s="31"/>
+      <c r="M35" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="N35" s="31"/>
+      <c r="O35" s="31"/>
+      <c r="P35" s="31"/>
+      <c r="Q35" s="31"/>
+      <c r="R35" s="31"/>
+      <c r="S35" s="31"/>
+      <c r="T35" s="31"/>
+      <c r="U35" s="31"/>
+      <c r="V35" s="32" t="s">
         <v>34</v>
-      </c>
-      <c r="B35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="17" t="n">
-        <v>152000</v>
-      </c>
-      <c r="I35" s="14"/>
-      <c r="J35" s="14"/>
-      <c r="K35" s="14"/>
-      <c r="L35" s="14"/>
-      <c r="M35" s="34" t="n">
-        <f aca="false">SUM(C35:L35)</f>
-        <v>152000</v>
-      </c>
-      <c r="N35" s="14"/>
-      <c r="O35" s="14"/>
-      <c r="P35" s="17" t="n">
-        <v>200000</v>
-      </c>
-      <c r="Q35" s="14"/>
-      <c r="R35" s="14"/>
-      <c r="S35" s="14"/>
-      <c r="T35" s="14"/>
-      <c r="U35" s="14"/>
-      <c r="V35" s="34" t="n">
-        <f aca="false">SUM(N35:U35)</f>
-        <v>200000</v>
       </c>
       <c r="W35" s="14"/>
       <c r="X35" s="14"/>
@@ -3095,7 +3087,7 @@
       <c r="F36" s="14"/>
       <c r="G36" s="14"/>
       <c r="H36" s="17" t="n">
-        <v>-96000</v>
+        <v>152000</v>
       </c>
       <c r="I36" s="14"/>
       <c r="J36" s="14"/>
@@ -3103,12 +3095,12 @@
       <c r="L36" s="14"/>
       <c r="M36" s="34" t="n">
         <f aca="false">SUM(C36:L36)</f>
-        <v>-96000</v>
+        <v>152000</v>
       </c>
       <c r="N36" s="14"/>
       <c r="O36" s="14"/>
       <c r="P36" s="17" t="n">
-        <v>-151000</v>
+        <v>200000</v>
       </c>
       <c r="Q36" s="14"/>
       <c r="R36" s="14"/>
@@ -3117,7 +3109,7 @@
       <c r="U36" s="14"/>
       <c r="V36" s="34" t="n">
         <f aca="false">SUM(N36:U36)</f>
-        <v>-151000</v>
+        <v>200000</v>
       </c>
       <c r="W36" s="14"/>
       <c r="X36" s="14"/>
@@ -3128,92 +3120,38 @@
       <c r="AC36" s="14"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="35" t="s">
+      <c r="A37" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="36" t="n">
-        <f aca="false">B35+B36</f>
-        <v>0</v>
-      </c>
-      <c r="C37" s="22" t="n">
-        <f aca="false">C35+C36</f>
-        <v>0</v>
-      </c>
-      <c r="D37" s="36" t="n">
-        <f aca="false">D35+D36</f>
-        <v>0</v>
-      </c>
-      <c r="E37" s="36" t="n">
-        <f aca="false">E35+E36</f>
-        <v>0</v>
-      </c>
-      <c r="F37" s="36" t="n">
-        <f aca="false">F35+F36</f>
-        <v>0</v>
-      </c>
-      <c r="G37" s="36" t="n">
-        <f aca="false">G35+G36</f>
-        <v>0</v>
-      </c>
-      <c r="H37" s="36" t="n">
-        <f aca="false">H35+H36</f>
-        <v>56000</v>
-      </c>
-      <c r="I37" s="36" t="n">
-        <f aca="false">I35+I36</f>
-        <v>0</v>
-      </c>
-      <c r="J37" s="36" t="n">
-        <f aca="false">J35+J36</f>
-        <v>0</v>
-      </c>
-      <c r="K37" s="36" t="n">
-        <f aca="false">K35+K36</f>
-        <v>0</v>
-      </c>
-      <c r="L37" s="36" t="n">
-        <f aca="false">L35+L36</f>
-        <v>0</v>
-      </c>
-      <c r="M37" s="37" t="n">
-        <f aca="false">M35+M36</f>
-        <v>56000</v>
-      </c>
-      <c r="N37" s="36" t="n">
-        <f aca="false">N35+N36</f>
-        <v>0</v>
-      </c>
-      <c r="O37" s="36" t="n">
-        <f aca="false">O35+O36</f>
-        <v>0</v>
-      </c>
-      <c r="P37" s="36" t="n">
-        <f aca="false">P35+P36</f>
-        <v>49000</v>
-      </c>
-      <c r="Q37" s="36" t="n">
-        <f aca="false">Q35+Q36</f>
-        <v>0</v>
-      </c>
-      <c r="R37" s="36" t="n">
-        <f aca="false">R35+R36</f>
-        <v>0</v>
-      </c>
-      <c r="S37" s="36" t="n">
-        <f aca="false">S35+S36</f>
-        <v>0</v>
-      </c>
-      <c r="T37" s="36" t="n">
-        <f aca="false">T35+T36</f>
-        <v>0</v>
-      </c>
-      <c r="U37" s="36" t="n">
-        <f aca="false">U35+U36</f>
-        <v>0</v>
-      </c>
-      <c r="V37" s="37" t="n">
-        <f aca="false">V35+V36</f>
-        <v>49000</v>
+      <c r="B37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="17" t="n">
+        <v>-96000</v>
+      </c>
+      <c r="I37" s="14"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14"/>
+      <c r="L37" s="14"/>
+      <c r="M37" s="34" t="n">
+        <f aca="false">SUM(C37:L37)</f>
+        <v>-96000</v>
+      </c>
+      <c r="N37" s="14"/>
+      <c r="O37" s="14"/>
+      <c r="P37" s="17" t="n">
+        <v>-151000</v>
+      </c>
+      <c r="Q37" s="14"/>
+      <c r="R37" s="14"/>
+      <c r="S37" s="14"/>
+      <c r="T37" s="14"/>
+      <c r="U37" s="14"/>
+      <c r="V37" s="34" t="n">
+        <f aca="false">SUM(N37:U37)</f>
+        <v>-151000</v>
       </c>
       <c r="W37" s="14"/>
       <c r="X37" s="14"/>
@@ -3224,29 +3162,93 @@
       <c r="AC37" s="14"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="38" t="s">
+      <c r="A38" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="14"/>
-      <c r="K38" s="14"/>
-      <c r="L38" s="14"/>
-      <c r="M38" s="39"/>
-      <c r="N38" s="14"/>
-      <c r="O38" s="14"/>
-      <c r="P38" s="14"/>
-      <c r="Q38" s="14"/>
-      <c r="R38" s="14"/>
-      <c r="S38" s="14"/>
-      <c r="T38" s="14"/>
-      <c r="U38" s="14"/>
-      <c r="V38" s="39"/>
+      <c r="B38" s="36" t="n">
+        <f aca="false">B36+B37</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="22" t="n">
+        <f aca="false">C36+C37</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="36" t="n">
+        <f aca="false">D36+D37</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="36" t="n">
+        <f aca="false">E36+E37</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="36" t="n">
+        <f aca="false">F36+F37</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="36" t="n">
+        <f aca="false">G36+G37</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="36" t="n">
+        <f aca="false">H36+H37</f>
+        <v>56000</v>
+      </c>
+      <c r="I38" s="36" t="n">
+        <f aca="false">I36+I37</f>
+        <v>0</v>
+      </c>
+      <c r="J38" s="36" t="n">
+        <f aca="false">J36+J37</f>
+        <v>0</v>
+      </c>
+      <c r="K38" s="36" t="n">
+        <f aca="false">K36+K37</f>
+        <v>0</v>
+      </c>
+      <c r="L38" s="36" t="n">
+        <f aca="false">L36+L37</f>
+        <v>0</v>
+      </c>
+      <c r="M38" s="37" t="n">
+        <f aca="false">M36+M37</f>
+        <v>56000</v>
+      </c>
+      <c r="N38" s="36" t="n">
+        <f aca="false">N36+N37</f>
+        <v>0</v>
+      </c>
+      <c r="O38" s="36" t="n">
+        <f aca="false">O36+O37</f>
+        <v>0</v>
+      </c>
+      <c r="P38" s="36" t="n">
+        <f aca="false">P36+P37</f>
+        <v>49000</v>
+      </c>
+      <c r="Q38" s="36" t="n">
+        <f aca="false">Q36+Q37</f>
+        <v>0</v>
+      </c>
+      <c r="R38" s="36" t="n">
+        <f aca="false">R36+R37</f>
+        <v>0</v>
+      </c>
+      <c r="S38" s="36" t="n">
+        <f aca="false">S36+S37</f>
+        <v>0</v>
+      </c>
+      <c r="T38" s="36" t="n">
+        <f aca="false">T36+T37</f>
+        <v>0</v>
+      </c>
+      <c r="U38" s="36" t="n">
+        <f aca="false">U36+U37</f>
+        <v>0</v>
+      </c>
+      <c r="V38" s="37" t="n">
+        <f aca="false">V36+V37</f>
+        <v>49000</v>
+      </c>
       <c r="W38" s="14"/>
       <c r="X38" s="14"/>
       <c r="Y38" s="14"/>
@@ -3256,7 +3258,7 @@
       <c r="AC38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="33" t="s">
+      <c r="A39" s="38" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="14"/>
@@ -3269,24 +3271,16 @@
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
-      <c r="M39" s="34" t="n">
-        <f aca="false">SUM(C39:L39)</f>
-        <v>0</v>
-      </c>
+      <c r="M39" s="39"/>
       <c r="N39" s="14"/>
       <c r="O39" s="14"/>
       <c r="P39" s="14"/>
       <c r="Q39" s="14"/>
       <c r="R39" s="14"/>
-      <c r="S39" s="17" t="n">
-        <v>-1200</v>
-      </c>
+      <c r="S39" s="14"/>
       <c r="T39" s="14"/>
       <c r="U39" s="14"/>
-      <c r="V39" s="34" t="n">
-        <f aca="false">SUM(N39:U39)</f>
-        <v>-1200</v>
-      </c>
+      <c r="V39" s="39"/>
       <c r="W39" s="14"/>
       <c r="X39" s="14"/>
       <c r="Y39" s="14"/>
@@ -3305,33 +3299,27 @@
       <c r="F40" s="14"/>
       <c r="G40" s="14"/>
       <c r="H40" s="14"/>
-      <c r="I40" s="17" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="J40" s="17" t="n">
-        <v>-2050</v>
-      </c>
+      <c r="I40" s="14"/>
+      <c r="J40" s="14"/>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
       <c r="M40" s="34" t="n">
         <f aca="false">SUM(C40:L40)</f>
-        <v>-4050</v>
+        <v>0</v>
       </c>
       <c r="N40" s="14"/>
       <c r="O40" s="14"/>
       <c r="P40" s="14"/>
       <c r="Q40" s="14"/>
-      <c r="R40" s="17" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="S40" s="14"/>
+      <c r="R40" s="14"/>
+      <c r="S40" s="17" t="n">
+        <v>-1200</v>
+      </c>
       <c r="T40" s="14"/>
-      <c r="U40" s="17" t="n">
-        <v>-2050</v>
-      </c>
+      <c r="U40" s="14"/>
       <c r="V40" s="34" t="n">
         <f aca="false">SUM(N40:U40)</f>
-        <v>-4050</v>
+        <v>-1200</v>
       </c>
       <c r="W40" s="14"/>
       <c r="X40" s="14"/>
@@ -3351,25 +3339,33 @@
       <c r="F41" s="14"/>
       <c r="G41" s="14"/>
       <c r="H41" s="14"/>
-      <c r="I41" s="14"/>
-      <c r="J41" s="14"/>
+      <c r="I41" s="17" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>-2050</v>
+      </c>
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
       <c r="M41" s="34" t="n">
         <f aca="false">SUM(C41:L41)</f>
-        <v>0</v>
+        <v>-4050</v>
       </c>
       <c r="N41" s="14"/>
       <c r="O41" s="14"/>
       <c r="P41" s="14"/>
       <c r="Q41" s="14"/>
-      <c r="R41" s="14"/>
+      <c r="R41" s="17" t="n">
+        <v>-2000</v>
+      </c>
       <c r="S41" s="14"/>
       <c r="T41" s="14"/>
-      <c r="U41" s="14"/>
+      <c r="U41" s="17" t="n">
+        <v>-2050</v>
+      </c>
       <c r="V41" s="34" t="n">
         <f aca="false">SUM(N41:U41)</f>
-        <v>0</v>
+        <v>-4050</v>
       </c>
       <c r="W41" s="14"/>
       <c r="X41" s="14"/>
@@ -3380,92 +3376,34 @@
       <c r="AC41" s="14"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="35" t="s">
+      <c r="A42" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="36" t="n">
-        <f aca="false">B37+SUM(B39:B41)</f>
-        <v>0</v>
-      </c>
-      <c r="C42" s="22" t="n">
-        <f aca="false">C37+SUM(C39:C41)</f>
-        <v>0</v>
-      </c>
-      <c r="D42" s="36" t="n">
-        <f aca="false">D37+SUM(D39:D41)</f>
-        <v>0</v>
-      </c>
-      <c r="E42" s="36" t="n">
-        <f aca="false">E37+SUM(E39:E41)</f>
-        <v>0</v>
-      </c>
-      <c r="F42" s="36" t="n">
-        <f aca="false">F37+SUM(F39:F41)</f>
-        <v>0</v>
-      </c>
-      <c r="G42" s="36" t="n">
-        <f aca="false">G37+SUM(G39:G41)</f>
-        <v>0</v>
-      </c>
-      <c r="H42" s="36" t="n">
-        <f aca="false">H37+SUM(H39:H41)</f>
-        <v>56000</v>
-      </c>
-      <c r="I42" s="36" t="n">
-        <f aca="false">I37+SUM(I39:I41)</f>
-        <v>-2000</v>
-      </c>
-      <c r="J42" s="36" t="n">
-        <f aca="false">J37+SUM(J39:J41)</f>
-        <v>-2050</v>
-      </c>
-      <c r="K42" s="36" t="n">
-        <f aca="false">K37+SUM(K39:K41)</f>
-        <v>0</v>
-      </c>
-      <c r="L42" s="36" t="n">
-        <f aca="false">L37+SUM(L39:L41)</f>
-        <v>0</v>
-      </c>
-      <c r="M42" s="37" t="n">
-        <f aca="false">M37+SUM(M39:M41)</f>
-        <v>51950</v>
-      </c>
-      <c r="N42" s="36" t="n">
-        <f aca="false">N37+SUM(N39:N41)</f>
-        <v>0</v>
-      </c>
-      <c r="O42" s="36" t="n">
-        <f aca="false">O37+SUM(O39:O41)</f>
-        <v>0</v>
-      </c>
-      <c r="P42" s="36" t="n">
-        <f aca="false">P37+SUM(P39:P41)</f>
-        <v>49000</v>
-      </c>
-      <c r="Q42" s="36" t="n">
-        <f aca="false">Q37+SUM(Q39:Q41)</f>
-        <v>0</v>
-      </c>
-      <c r="R42" s="36" t="n">
-        <f aca="false">R37+SUM(R39:R41)</f>
-        <v>-2000</v>
-      </c>
-      <c r="S42" s="36" t="n">
-        <f aca="false">S37+SUM(S39:S41)</f>
-        <v>-1200</v>
-      </c>
-      <c r="T42" s="36" t="n">
-        <f aca="false">T37+SUM(T39:T41)</f>
-        <v>0</v>
-      </c>
-      <c r="U42" s="36" t="n">
-        <f aca="false">U37+SUM(U39:U41)</f>
-        <v>-2050</v>
-      </c>
-      <c r="V42" s="37" t="n">
-        <f aca="false">V37+SUM(V39:V41)</f>
-        <v>43750</v>
+      <c r="B42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="L42" s="14"/>
+      <c r="M42" s="34" t="n">
+        <f aca="false">SUM(C42:L42)</f>
+        <v>0</v>
+      </c>
+      <c r="N42" s="14"/>
+      <c r="O42" s="14"/>
+      <c r="P42" s="14"/>
+      <c r="Q42" s="14"/>
+      <c r="R42" s="14"/>
+      <c r="S42" s="14"/>
+      <c r="T42" s="14"/>
+      <c r="U42" s="14"/>
+      <c r="V42" s="34" t="n">
+        <f aca="false">SUM(N42:U42)</f>
+        <v>0</v>
       </c>
       <c r="W42" s="14"/>
       <c r="X42" s="14"/>
@@ -3476,38 +3414,92 @@
       <c r="AC42" s="14"/>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="33" t="s">
+      <c r="A43" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="17" t="n">
-        <v>-500</v>
-      </c>
-      <c r="K43" s="14"/>
-      <c r="L43" s="14"/>
-      <c r="M43" s="34" t="n">
-        <f aca="false">SUM(C43:L43)</f>
-        <v>-500</v>
-      </c>
-      <c r="N43" s="14"/>
-      <c r="O43" s="14"/>
-      <c r="P43" s="14"/>
-      <c r="Q43" s="14"/>
-      <c r="R43" s="14"/>
-      <c r="S43" s="14"/>
-      <c r="T43" s="17" t="n">
-        <v>-500</v>
-      </c>
-      <c r="U43" s="14"/>
-      <c r="V43" s="34" t="n">
-        <f aca="false">SUM(N43:U43)</f>
-        <v>-500</v>
+      <c r="B43" s="36" t="n">
+        <f aca="false">B38+SUM(B40:B42)</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="22" t="n">
+        <f aca="false">C38+SUM(C40:C42)</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="36" t="n">
+        <f aca="false">D38+SUM(D40:D42)</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="36" t="n">
+        <f aca="false">E38+SUM(E40:E42)</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="36" t="n">
+        <f aca="false">F38+SUM(F40:F42)</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="36" t="n">
+        <f aca="false">G38+SUM(G40:G42)</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="36" t="n">
+        <f aca="false">H38+SUM(H40:H42)</f>
+        <v>56000</v>
+      </c>
+      <c r="I43" s="36" t="n">
+        <f aca="false">I38+SUM(I40:I42)</f>
+        <v>-2000</v>
+      </c>
+      <c r="J43" s="36" t="n">
+        <f aca="false">J38+SUM(J40:J42)</f>
+        <v>-2050</v>
+      </c>
+      <c r="K43" s="36" t="n">
+        <f aca="false">K38+SUM(K40:K42)</f>
+        <v>0</v>
+      </c>
+      <c r="L43" s="36" t="n">
+        <f aca="false">L38+SUM(L40:L42)</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="37" t="n">
+        <f aca="false">M38+SUM(M40:M42)</f>
+        <v>51950</v>
+      </c>
+      <c r="N43" s="36" t="n">
+        <f aca="false">N38+SUM(N40:N42)</f>
+        <v>0</v>
+      </c>
+      <c r="O43" s="36" t="n">
+        <f aca="false">O38+SUM(O40:O42)</f>
+        <v>0</v>
+      </c>
+      <c r="P43" s="36" t="n">
+        <f aca="false">P38+SUM(P40:P42)</f>
+        <v>49000</v>
+      </c>
+      <c r="Q43" s="36" t="n">
+        <f aca="false">Q38+SUM(Q40:Q42)</f>
+        <v>0</v>
+      </c>
+      <c r="R43" s="36" t="n">
+        <f aca="false">R38+SUM(R40:R42)</f>
+        <v>-2000</v>
+      </c>
+      <c r="S43" s="36" t="n">
+        <f aca="false">S38+SUM(S40:S42)</f>
+        <v>-1200</v>
+      </c>
+      <c r="T43" s="36" t="n">
+        <f aca="false">T38+SUM(T40:T42)</f>
+        <v>0</v>
+      </c>
+      <c r="U43" s="36" t="n">
+        <f aca="false">U38+SUM(U40:U42)</f>
+        <v>-2050</v>
+      </c>
+      <c r="V43" s="37" t="n">
+        <f aca="false">V38+SUM(V40:V42)</f>
+        <v>43750</v>
       </c>
       <c r="W43" s="14"/>
       <c r="X43" s="14"/>
@@ -3518,92 +3510,38 @@
       <c r="AC43" s="14"/>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="35" t="s">
+      <c r="A44" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="36" t="n">
-        <f aca="false">B42+B43</f>
-        <v>0</v>
-      </c>
-      <c r="C44" s="22" t="n">
-        <f aca="false">C42+C43</f>
-        <v>0</v>
-      </c>
-      <c r="D44" s="36" t="n">
-        <f aca="false">D42+D43</f>
-        <v>0</v>
-      </c>
-      <c r="E44" s="36" t="n">
-        <f aca="false">E42+E43</f>
-        <v>0</v>
-      </c>
-      <c r="F44" s="36" t="n">
-        <f aca="false">F42+F43</f>
-        <v>0</v>
-      </c>
-      <c r="G44" s="36" t="n">
-        <f aca="false">G42+G43</f>
-        <v>0</v>
-      </c>
-      <c r="H44" s="36" t="n">
-        <f aca="false">H42+H43</f>
-        <v>56000</v>
-      </c>
-      <c r="I44" s="36" t="n">
-        <f aca="false">I42+I43</f>
-        <v>-2000</v>
-      </c>
-      <c r="J44" s="36" t="n">
-        <f aca="false">J42+J43</f>
-        <v>-2550</v>
-      </c>
-      <c r="K44" s="36" t="n">
-        <f aca="false">K42+K43</f>
-        <v>0</v>
-      </c>
-      <c r="L44" s="36" t="n">
-        <f aca="false">L42+L43</f>
-        <v>0</v>
-      </c>
-      <c r="M44" s="37" t="n">
-        <f aca="false">M42+M43</f>
-        <v>51450</v>
-      </c>
-      <c r="N44" s="36" t="n">
-        <f aca="false">N42+N43</f>
-        <v>0</v>
-      </c>
-      <c r="O44" s="36" t="n">
-        <f aca="false">O42+O43</f>
-        <v>0</v>
-      </c>
-      <c r="P44" s="36" t="n">
-        <f aca="false">P42+P43</f>
-        <v>49000</v>
-      </c>
-      <c r="Q44" s="36" t="n">
-        <f aca="false">Q42+Q43</f>
-        <v>0</v>
-      </c>
-      <c r="R44" s="36" t="n">
-        <f aca="false">R42+R43</f>
-        <v>-2000</v>
-      </c>
-      <c r="S44" s="36" t="n">
-        <f aca="false">S42+S43</f>
-        <v>-1200</v>
-      </c>
-      <c r="T44" s="36" t="n">
-        <f aca="false">T42+T43</f>
+      <c r="B44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="17" t="n">
         <v>-500</v>
       </c>
-      <c r="U44" s="36" t="n">
-        <f aca="false">U42+U43</f>
-        <v>-2050</v>
-      </c>
-      <c r="V44" s="37" t="n">
-        <f aca="false">V42+V43</f>
-        <v>43250</v>
+      <c r="K44" s="14"/>
+      <c r="L44" s="14"/>
+      <c r="M44" s="34" t="n">
+        <f aca="false">SUM(C44:L44)</f>
+        <v>-500</v>
+      </c>
+      <c r="N44" s="14"/>
+      <c r="O44" s="14"/>
+      <c r="P44" s="14"/>
+      <c r="Q44" s="14"/>
+      <c r="R44" s="14"/>
+      <c r="S44" s="14"/>
+      <c r="T44" s="17" t="n">
+        <v>-500</v>
+      </c>
+      <c r="U44" s="14"/>
+      <c r="V44" s="34" t="n">
+        <f aca="false">SUM(N44:U44)</f>
+        <v>-500</v>
       </c>
       <c r="W44" s="14"/>
       <c r="X44" s="14"/>
@@ -3614,40 +3552,92 @@
       <c r="AC44" s="14"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="33" t="s">
+      <c r="A45" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="14"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="19" t="n">
-        <f aca="false">-0.3*M44</f>
-        <v>-15435</v>
-      </c>
-      <c r="L45" s="14"/>
-      <c r="M45" s="34" t="n">
-        <f aca="false">SUM(C45:L45)</f>
-        <v>-15435</v>
-      </c>
-      <c r="N45" s="14"/>
-      <c r="O45" s="14"/>
-      <c r="P45" s="14"/>
-      <c r="Q45" s="14"/>
-      <c r="R45" s="14"/>
-      <c r="S45" s="14"/>
-      <c r="T45" s="14"/>
-      <c r="U45" s="19" t="n">
-        <f aca="false">-0.3*V44</f>
-        <v>-12975</v>
-      </c>
-      <c r="V45" s="34" t="n">
-        <f aca="false">SUM(N45:U45)</f>
-        <v>-12975</v>
+      <c r="B45" s="36" t="n">
+        <f aca="false">B43+B44</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="22" t="n">
+        <f aca="false">C43+C44</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="36" t="n">
+        <f aca="false">D43+D44</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="36" t="n">
+        <f aca="false">E43+E44</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="36" t="n">
+        <f aca="false">F43+F44</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="36" t="n">
+        <f aca="false">G43+G44</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="36" t="n">
+        <f aca="false">H43+H44</f>
+        <v>56000</v>
+      </c>
+      <c r="I45" s="36" t="n">
+        <f aca="false">I43+I44</f>
+        <v>-2000</v>
+      </c>
+      <c r="J45" s="36" t="n">
+        <f aca="false">J43+J44</f>
+        <v>-2550</v>
+      </c>
+      <c r="K45" s="36" t="n">
+        <f aca="false">K43+K44</f>
+        <v>0</v>
+      </c>
+      <c r="L45" s="36" t="n">
+        <f aca="false">L43+L44</f>
+        <v>0</v>
+      </c>
+      <c r="M45" s="37" t="n">
+        <f aca="false">M43+M44</f>
+        <v>51450</v>
+      </c>
+      <c r="N45" s="36" t="n">
+        <f aca="false">N43+N44</f>
+        <v>0</v>
+      </c>
+      <c r="O45" s="36" t="n">
+        <f aca="false">O43+O44</f>
+        <v>0</v>
+      </c>
+      <c r="P45" s="36" t="n">
+        <f aca="false">P43+P44</f>
+        <v>49000</v>
+      </c>
+      <c r="Q45" s="36" t="n">
+        <f aca="false">Q43+Q44</f>
+        <v>0</v>
+      </c>
+      <c r="R45" s="36" t="n">
+        <f aca="false">R43+R44</f>
+        <v>-2000</v>
+      </c>
+      <c r="S45" s="36" t="n">
+        <f aca="false">S43+S44</f>
+        <v>-1200</v>
+      </c>
+      <c r="T45" s="36" t="n">
+        <f aca="false">T43+T44</f>
+        <v>-500</v>
+      </c>
+      <c r="U45" s="36" t="n">
+        <f aca="false">U43+U44</f>
+        <v>-2050</v>
+      </c>
+      <c r="V45" s="37" t="n">
+        <f aca="false">V43+V44</f>
+        <v>43250</v>
       </c>
       <c r="W45" s="14"/>
       <c r="X45" s="14"/>
@@ -3658,92 +3648,40 @@
       <c r="AC45" s="14"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="20" t="s">
+      <c r="A46" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="21" t="n">
-        <f aca="false">B44+B45</f>
-        <v>0</v>
-      </c>
-      <c r="C46" s="22" t="n">
-        <f aca="false">C44+C45</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="21" t="n">
-        <f aca="false">D44+D45</f>
-        <v>0</v>
-      </c>
-      <c r="E46" s="21" t="n">
-        <f aca="false">E44+E45</f>
-        <v>0</v>
-      </c>
-      <c r="F46" s="21" t="n">
-        <f aca="false">F44+F45</f>
-        <v>0</v>
-      </c>
-      <c r="G46" s="21" t="n">
-        <f aca="false">G44+G45</f>
-        <v>0</v>
-      </c>
-      <c r="H46" s="21" t="n">
-        <f aca="false">H44+H45</f>
-        <v>56000</v>
-      </c>
-      <c r="I46" s="21" t="n">
-        <f aca="false">I44+I45</f>
-        <v>-2000</v>
-      </c>
-      <c r="J46" s="21" t="n">
-        <f aca="false">J44+J45</f>
-        <v>-2550</v>
-      </c>
-      <c r="K46" s="21" t="n">
-        <f aca="false">K44+K45</f>
+      <c r="B46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="19" t="n">
+        <f aca="false">-0.3*M45</f>
         <v>-15435</v>
       </c>
-      <c r="L46" s="21" t="n">
-        <f aca="false">L44+L45</f>
-        <v>0</v>
-      </c>
-      <c r="M46" s="21" t="n">
-        <f aca="false">M44+M45</f>
-        <v>36015</v>
-      </c>
-      <c r="N46" s="21" t="n">
-        <f aca="false">N44+N45</f>
-        <v>0</v>
-      </c>
-      <c r="O46" s="21" t="n">
-        <f aca="false">O44+O45</f>
-        <v>0</v>
-      </c>
-      <c r="P46" s="21" t="n">
-        <f aca="false">P44+P45</f>
-        <v>49000</v>
-      </c>
-      <c r="Q46" s="21" t="n">
-        <f aca="false">Q44+Q45</f>
-        <v>0</v>
-      </c>
-      <c r="R46" s="21" t="n">
-        <f aca="false">R44+R45</f>
-        <v>-2000</v>
-      </c>
-      <c r="S46" s="21" t="n">
-        <f aca="false">S44+S45</f>
-        <v>-1200</v>
-      </c>
-      <c r="T46" s="21" t="n">
-        <f aca="false">T44+T45</f>
-        <v>-500</v>
-      </c>
-      <c r="U46" s="21" t="n">
-        <f aca="false">U44+U45</f>
-        <v>-15025</v>
-      </c>
-      <c r="V46" s="21" t="n">
-        <f aca="false">V44+V45</f>
-        <v>30275</v>
+      <c r="L46" s="14"/>
+      <c r="M46" s="34" t="n">
+        <f aca="false">SUM(C46:L46)</f>
+        <v>-15435</v>
+      </c>
+      <c r="N46" s="14"/>
+      <c r="O46" s="14"/>
+      <c r="P46" s="14"/>
+      <c r="Q46" s="14"/>
+      <c r="R46" s="14"/>
+      <c r="S46" s="14"/>
+      <c r="T46" s="14"/>
+      <c r="U46" s="19" t="n">
+        <f aca="false">-0.3*V45</f>
+        <v>-12975</v>
+      </c>
+      <c r="V46" s="34" t="n">
+        <f aca="false">SUM(N46:U46)</f>
+        <v>-12975</v>
       </c>
       <c r="W46" s="14"/>
       <c r="X46" s="14"/>
@@ -3753,62 +3691,133 @@
       <c r="AB46" s="14"/>
       <c r="AC46" s="14"/>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="30" t="s">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="40"/>
-      <c r="D49" s="40"/>
-      <c r="E49" s="40"/>
-      <c r="F49" s="40"/>
-      <c r="G49" s="40"/>
-      <c r="H49" s="40"/>
-      <c r="I49" s="40"/>
-      <c r="J49" s="40"/>
-      <c r="K49" s="40"/>
-      <c r="L49" s="41"/>
-      <c r="M49" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="N49" s="31"/>
-      <c r="O49" s="31"/>
-      <c r="P49" s="31"/>
-      <c r="Q49" s="31"/>
-      <c r="R49" s="31"/>
-      <c r="S49" s="31"/>
-      <c r="T49" s="31"/>
-      <c r="U49" s="31"/>
-      <c r="V49" s="32" t="s">
+      <c r="B47" s="21" t="n">
+        <f aca="false">B45+B46</f>
+        <v>0</v>
+      </c>
+      <c r="C47" s="22" t="n">
+        <f aca="false">C45+C46</f>
+        <v>0</v>
+      </c>
+      <c r="D47" s="21" t="n">
+        <f aca="false">D45+D46</f>
+        <v>0</v>
+      </c>
+      <c r="E47" s="21" t="n">
+        <f aca="false">E45+E46</f>
+        <v>0</v>
+      </c>
+      <c r="F47" s="21" t="n">
+        <f aca="false">F45+F46</f>
+        <v>0</v>
+      </c>
+      <c r="G47" s="21" t="n">
+        <f aca="false">G45+G46</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="21" t="n">
+        <f aca="false">H45+H46</f>
+        <v>56000</v>
+      </c>
+      <c r="I47" s="21" t="n">
+        <f aca="false">I45+I46</f>
+        <v>-2000</v>
+      </c>
+      <c r="J47" s="21" t="n">
+        <f aca="false">J45+J46</f>
+        <v>-2550</v>
+      </c>
+      <c r="K47" s="21" t="n">
+        <f aca="false">K45+K46</f>
+        <v>-15435</v>
+      </c>
+      <c r="L47" s="21" t="n">
+        <f aca="false">L45+L46</f>
+        <v>0</v>
+      </c>
+      <c r="M47" s="21" t="n">
+        <f aca="false">M45+M46</f>
+        <v>36015</v>
+      </c>
+      <c r="N47" s="21" t="n">
+        <f aca="false">N45+N46</f>
+        <v>0</v>
+      </c>
+      <c r="O47" s="21" t="n">
+        <f aca="false">O45+O46</f>
+        <v>0</v>
+      </c>
+      <c r="P47" s="21" t="n">
+        <f aca="false">P45+P46</f>
+        <v>49000</v>
+      </c>
+      <c r="Q47" s="21" t="n">
+        <f aca="false">Q45+Q46</f>
+        <v>0</v>
+      </c>
+      <c r="R47" s="21" t="n">
+        <f aca="false">R45+R46</f>
+        <v>-2000</v>
+      </c>
+      <c r="S47" s="21" t="n">
+        <f aca="false">S45+S46</f>
+        <v>-1200</v>
+      </c>
+      <c r="T47" s="21" t="n">
+        <f aca="false">T45+T46</f>
+        <v>-500</v>
+      </c>
+      <c r="U47" s="21" t="n">
+        <f aca="false">U45+U46</f>
+        <v>-15025</v>
+      </c>
+      <c r="V47" s="21" t="n">
+        <f aca="false">V45+V46</f>
+        <v>30275</v>
+      </c>
+      <c r="W47" s="14"/>
+      <c r="X47" s="14"/>
+      <c r="Y47" s="14"/>
+      <c r="Z47" s="14"/>
+      <c r="AA47" s="14"/>
+      <c r="AB47" s="14"/>
+      <c r="AC47" s="14"/>
+    </row>
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="B50" s="40"/>
+      <c r="D50" s="40"/>
+      <c r="E50" s="40"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="40"/>
+      <c r="I50" s="40"/>
+      <c r="J50" s="40"/>
+      <c r="K50" s="40"/>
+      <c r="L50" s="41"/>
+      <c r="M50" s="32" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="42" t="s">
-        <v>47</v>
-      </c>
-      <c r="B50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
-      <c r="L50" s="14"/>
-      <c r="M50" s="43"/>
-      <c r="N50" s="14"/>
-      <c r="O50" s="14"/>
-      <c r="P50" s="14"/>
-      <c r="Q50" s="14"/>
-      <c r="R50" s="14"/>
-      <c r="S50" s="14"/>
-      <c r="T50" s="14"/>
-      <c r="U50" s="14"/>
-      <c r="V50" s="43"/>
+      <c r="N50" s="31"/>
+      <c r="O50" s="31"/>
+      <c r="P50" s="31"/>
+      <c r="Q50" s="31"/>
+      <c r="R50" s="31"/>
+      <c r="S50" s="31"/>
+      <c r="T50" s="31"/>
+      <c r="U50" s="31"/>
+      <c r="V50" s="32" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="33" t="s">
+      <c r="A51" s="42" t="s">
         <v>48</v>
       </c>
       <c r="B51" s="14"/>
@@ -3816,273 +3825,268 @@
       <c r="E51" s="14"/>
       <c r="F51" s="14"/>
       <c r="G51" s="14"/>
-      <c r="H51" s="17" t="n">
-        <v>122000</v>
-      </c>
+      <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14"/>
       <c r="K51" s="14"/>
       <c r="L51" s="14"/>
-      <c r="M51" s="44" t="n">
-        <f aca="false">SUM(C51:L51)</f>
-        <v>122000</v>
-      </c>
-      <c r="N51" s="17" t="n">
-        <v>50000</v>
-      </c>
+      <c r="M51" s="43"/>
+      <c r="N51" s="14"/>
       <c r="O51" s="14"/>
-      <c r="P51" s="17" t="n">
-        <v>156000</v>
-      </c>
-      <c r="Q51" s="17" t="n">
-        <v>250</v>
-      </c>
+      <c r="P51" s="14"/>
+      <c r="Q51" s="14"/>
       <c r="R51" s="14"/>
       <c r="S51" s="14"/>
       <c r="T51" s="14"/>
       <c r="U51" s="14"/>
-      <c r="V51" s="44" t="n">
-        <f aca="false">SUM(N51:U51)</f>
-        <v>206250</v>
-      </c>
+      <c r="V51" s="43"/>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="35" t="s">
+      <c r="A52" s="33" t="s">
         <v>49</v>
       </c>
       <c r="B52" s="14"/>
       <c r="D52" s="14"/>
       <c r="E52" s="14"/>
-      <c r="F52" s="17" t="n">
-        <v>-100000</v>
-      </c>
+      <c r="F52" s="14"/>
       <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
+      <c r="H52" s="17" t="n">
+        <v>122000</v>
+      </c>
       <c r="I52" s="14"/>
       <c r="J52" s="14"/>
       <c r="K52" s="14"/>
       <c r="L52" s="14"/>
       <c r="M52" s="44" t="n">
         <f aca="false">SUM(C52:L52)</f>
-        <v>-100000</v>
-      </c>
-      <c r="N52" s="14"/>
-      <c r="O52" s="17" t="n">
-        <v>-155000</v>
-      </c>
-      <c r="P52" s="14"/>
-      <c r="Q52" s="14"/>
+        <v>122000</v>
+      </c>
+      <c r="N52" s="17" t="n">
+        <v>50000</v>
+      </c>
+      <c r="O52" s="14"/>
+      <c r="P52" s="17" t="n">
+        <v>156000</v>
+      </c>
+      <c r="Q52" s="17" t="n">
+        <v>250</v>
+      </c>
       <c r="R52" s="14"/>
       <c r="S52" s="14"/>
       <c r="T52" s="14"/>
       <c r="U52" s="14"/>
       <c r="V52" s="44" t="n">
         <f aca="false">SUM(N52:U52)</f>
-        <v>-155000</v>
+        <v>206250</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="38" t="s">
+      <c r="A53" s="35" t="s">
         <v>50</v>
       </c>
       <c r="B53" s="14"/>
       <c r="D53" s="14"/>
-      <c r="E53" s="17" t="n">
-        <v>-9000</v>
-      </c>
-      <c r="F53" s="14"/>
-      <c r="G53" s="17" t="n">
-        <v>-1200</v>
-      </c>
+      <c r="E53" s="14"/>
+      <c r="F53" s="17" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="G53" s="14"/>
       <c r="H53" s="14"/>
-      <c r="I53" s="17" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="I53" s="14"/>
       <c r="J53" s="14"/>
       <c r="K53" s="14"/>
       <c r="L53" s="14"/>
       <c r="M53" s="44" t="n">
         <f aca="false">SUM(C53:L53)</f>
-        <v>-11200</v>
-      </c>
-      <c r="N53" s="17" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="O53" s="14"/>
+        <v>-100000</v>
+      </c>
+      <c r="N53" s="14"/>
+      <c r="O53" s="17" t="n">
+        <v>-155000</v>
+      </c>
       <c r="P53" s="14"/>
       <c r="Q53" s="14"/>
-      <c r="R53" s="17" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="R53" s="14"/>
       <c r="S53" s="14"/>
       <c r="T53" s="14"/>
       <c r="U53" s="14"/>
       <c r="V53" s="44" t="n">
         <f aca="false">SUM(N53:U53)</f>
-        <v>-2000</v>
+        <v>-155000</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="33" t="s">
+      <c r="A54" s="38" t="s">
         <v>51</v>
       </c>
       <c r="B54" s="14"/>
       <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
+      <c r="E54" s="17" t="n">
+        <v>-9000</v>
+      </c>
       <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
+      <c r="G54" s="17" t="n">
+        <v>-1200</v>
+      </c>
       <c r="H54" s="14"/>
-      <c r="I54" s="14"/>
+      <c r="I54" s="17" t="n">
+        <v>-1000</v>
+      </c>
       <c r="J54" s="14"/>
       <c r="K54" s="14"/>
       <c r="L54" s="14"/>
       <c r="M54" s="44" t="n">
         <f aca="false">SUM(C54:L54)</f>
-        <v>0</v>
-      </c>
-      <c r="N54" s="14"/>
+        <v>-11200</v>
+      </c>
+      <c r="N54" s="17" t="n">
+        <v>-1000</v>
+      </c>
       <c r="O54" s="14"/>
       <c r="P54" s="14"/>
       <c r="Q54" s="14"/>
-      <c r="R54" s="14"/>
+      <c r="R54" s="17" t="n">
+        <v>-1000</v>
+      </c>
       <c r="S54" s="14"/>
-      <c r="T54" s="17" t="n">
+      <c r="T54" s="14"/>
+      <c r="U54" s="14"/>
+      <c r="V54" s="44" t="n">
+        <f aca="false">SUM(N54:U54)</f>
+        <v>-2000</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="B55" s="14"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="14"/>
+      <c r="G55" s="14"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="14"/>
+      <c r="K55" s="14"/>
+      <c r="L55" s="14"/>
+      <c r="M55" s="44" t="n">
+        <f aca="false">SUM(C55:L55)</f>
+        <v>0</v>
+      </c>
+      <c r="N55" s="14"/>
+      <c r="O55" s="14"/>
+      <c r="P55" s="14"/>
+      <c r="Q55" s="14"/>
+      <c r="R55" s="14"/>
+      <c r="S55" s="14"/>
+      <c r="T55" s="17" t="n">
         <v>-1000</v>
       </c>
-      <c r="U54" s="19" t="n">
+      <c r="U55" s="19" t="n">
         <f aca="false">-M20</f>
         <v>-15435</v>
       </c>
-      <c r="V54" s="44" t="n">
-        <f aca="false">SUM(N54:U54)</f>
+      <c r="V55" s="44" t="n">
+        <f aca="false">SUM(N55:U55)</f>
         <v>-16435</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="42" t="s">
-        <v>52</v>
-      </c>
-      <c r="B55" s="45"/>
-      <c r="D55" s="45"/>
-      <c r="E55" s="45"/>
-      <c r="F55" s="45"/>
-      <c r="G55" s="45"/>
-      <c r="H55" s="45"/>
-      <c r="I55" s="45"/>
-      <c r="J55" s="45"/>
-      <c r="K55" s="45"/>
-      <c r="L55" s="45"/>
-      <c r="M55" s="46"/>
-      <c r="N55" s="45"/>
-      <c r="O55" s="45"/>
-      <c r="P55" s="45"/>
-      <c r="Q55" s="45"/>
-      <c r="R55" s="45"/>
-      <c r="S55" s="45"/>
-      <c r="T55" s="45"/>
-      <c r="U55" s="45"/>
-      <c r="V55" s="46"/>
-    </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="33" t="s">
+      <c r="A56" s="42" t="s">
         <v>53</v>
       </c>
-      <c r="B56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="17" t="n">
+      <c r="B56" s="45"/>
+      <c r="D56" s="45"/>
+      <c r="E56" s="45"/>
+      <c r="F56" s="45"/>
+      <c r="G56" s="45"/>
+      <c r="H56" s="45"/>
+      <c r="I56" s="45"/>
+      <c r="J56" s="45"/>
+      <c r="K56" s="45"/>
+      <c r="L56" s="45"/>
+      <c r="M56" s="46"/>
+      <c r="N56" s="45"/>
+      <c r="O56" s="45"/>
+      <c r="P56" s="45"/>
+      <c r="Q56" s="45"/>
+      <c r="R56" s="45"/>
+      <c r="S56" s="45"/>
+      <c r="T56" s="45"/>
+      <c r="U56" s="45"/>
+      <c r="V56" s="46"/>
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="17" t="n">
         <v>-13200</v>
       </c>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="14"/>
-      <c r="J56" s="14"/>
-      <c r="K56" s="14"/>
-      <c r="L56" s="14"/>
-      <c r="M56" s="44" t="n">
-        <f aca="false">SUM(C56:L56)</f>
+      <c r="F57" s="14"/>
+      <c r="G57" s="14"/>
+      <c r="H57" s="14"/>
+      <c r="I57" s="14"/>
+      <c r="J57" s="14"/>
+      <c r="K57" s="14"/>
+      <c r="L57" s="14"/>
+      <c r="M57" s="44" t="n">
+        <f aca="false">SUM(C57:L57)</f>
         <v>-13200</v>
       </c>
-      <c r="N56" s="14"/>
-      <c r="O56" s="14"/>
-      <c r="P56" s="14"/>
-      <c r="Q56" s="14"/>
-      <c r="R56" s="14"/>
-      <c r="S56" s="14"/>
-      <c r="T56" s="14"/>
-      <c r="U56" s="14"/>
-      <c r="V56" s="44" t="n">
-        <f aca="false">SUM(N56:U56)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47" t="s">
-        <v>54</v>
-      </c>
-      <c r="B57" s="48"/>
-      <c r="D57" s="48"/>
-      <c r="E57" s="48"/>
-      <c r="F57" s="48"/>
-      <c r="G57" s="48"/>
-      <c r="H57" s="48"/>
-      <c r="I57" s="48"/>
-      <c r="J57" s="48"/>
-      <c r="K57" s="48"/>
-      <c r="L57" s="48"/>
-      <c r="M57" s="49" t="n">
-        <f aca="false">SUM(C57:L57)</f>
-        <v>0</v>
-      </c>
-      <c r="N57" s="48"/>
-      <c r="O57" s="48"/>
-      <c r="P57" s="48"/>
-      <c r="Q57" s="48"/>
-      <c r="R57" s="48"/>
-      <c r="S57" s="48"/>
-      <c r="T57" s="48"/>
-      <c r="U57" s="48"/>
-      <c r="V57" s="49" t="n">
+      <c r="N57" s="14"/>
+      <c r="O57" s="14"/>
+      <c r="P57" s="14"/>
+      <c r="Q57" s="14"/>
+      <c r="R57" s="14"/>
+      <c r="S57" s="14"/>
+      <c r="T57" s="14"/>
+      <c r="U57" s="14"/>
+      <c r="V57" s="44" t="n">
         <f aca="false">SUM(N57:U57)</f>
         <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="50" t="s">
+      <c r="A58" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="B58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="14"/>
-      <c r="K58" s="14"/>
-      <c r="L58" s="14"/>
-      <c r="M58" s="43"/>
-      <c r="N58" s="14"/>
-      <c r="O58" s="14"/>
-      <c r="P58" s="14"/>
-      <c r="Q58" s="14"/>
-      <c r="R58" s="14"/>
-      <c r="S58" s="14"/>
-      <c r="T58" s="14"/>
-      <c r="U58" s="14"/>
-      <c r="V58" s="43"/>
+      <c r="B58" s="48"/>
+      <c r="D58" s="48"/>
+      <c r="E58" s="48"/>
+      <c r="F58" s="48"/>
+      <c r="G58" s="48"/>
+      <c r="H58" s="48"/>
+      <c r="I58" s="48"/>
+      <c r="J58" s="48"/>
+      <c r="K58" s="48"/>
+      <c r="L58" s="48"/>
+      <c r="M58" s="49" t="n">
+        <f aca="false">SUM(C58:L58)</f>
+        <v>0</v>
+      </c>
+      <c r="N58" s="48"/>
+      <c r="O58" s="48"/>
+      <c r="P58" s="48"/>
+      <c r="Q58" s="48"/>
+      <c r="R58" s="48"/>
+      <c r="S58" s="48"/>
+      <c r="T58" s="48"/>
+      <c r="U58" s="48"/>
+      <c r="V58" s="49" t="n">
+        <f aca="false">SUM(N58:U58)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="35" t="s">
+      <c r="A59" s="50" t="s">
         <v>56</v>
       </c>
       <c r="B59" s="14"/>
-      <c r="C59" s="16" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D59" s="17" t="n">
-        <v>50000</v>
-      </c>
+      <c r="D59" s="14"/>
       <c r="E59" s="14"/>
       <c r="F59" s="14"/>
       <c r="G59" s="14"/>
@@ -4091,10 +4095,7 @@
       <c r="J59" s="14"/>
       <c r="K59" s="14"/>
       <c r="L59" s="14"/>
-      <c r="M59" s="44" t="n">
-        <f aca="false">SUM(C59:L59)</f>
-        <v>130000</v>
-      </c>
+      <c r="M59" s="43"/>
       <c r="N59" s="14"/>
       <c r="O59" s="14"/>
       <c r="P59" s="14"/>
@@ -4103,17 +4104,19 @@
       <c r="S59" s="14"/>
       <c r="T59" s="14"/>
       <c r="U59" s="14"/>
-      <c r="V59" s="44" t="n">
-        <f aca="false">SUM(N59:U59)</f>
-        <v>0</v>
-      </c>
+      <c r="V59" s="43"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="33" t="s">
+      <c r="A60" s="35" t="s">
         <v>57</v>
       </c>
       <c r="B60" s="14"/>
-      <c r="D60" s="14"/>
+      <c r="C60" s="16" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D60" s="17" t="n">
+        <v>50000</v>
+      </c>
       <c r="E60" s="14"/>
       <c r="F60" s="14"/>
       <c r="G60" s="14"/>
@@ -4124,282 +4127,313 @@
       <c r="L60" s="14"/>
       <c r="M60" s="44" t="n">
         <f aca="false">SUM(C60:L60)</f>
-        <v>0</v>
-      </c>
-      <c r="N60" s="19" t="n">
-        <f aca="false">-M22</f>
-        <v>-14406</v>
-      </c>
+        <v>130000</v>
+      </c>
+      <c r="N60" s="14"/>
       <c r="O60" s="14"/>
       <c r="P60" s="14"/>
       <c r="Q60" s="14"/>
       <c r="R60" s="14"/>
       <c r="S60" s="14"/>
-      <c r="T60" s="17" t="n">
-        <v>-50000</v>
-      </c>
+      <c r="T60" s="14"/>
       <c r="U60" s="14"/>
       <c r="V60" s="44" t="n">
         <f aca="false">SUM(N60:U60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="B61" s="14"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="14"/>
+      <c r="G61" s="14"/>
+      <c r="H61" s="14"/>
+      <c r="I61" s="14"/>
+      <c r="J61" s="14"/>
+      <c r="K61" s="14"/>
+      <c r="L61" s="14"/>
+      <c r="M61" s="44" t="n">
+        <f aca="false">SUM(C61:L61)</f>
+        <v>0</v>
+      </c>
+      <c r="N61" s="19" t="n">
+        <f aca="false">-M22</f>
+        <v>-14406</v>
+      </c>
+      <c r="O61" s="14"/>
+      <c r="P61" s="14"/>
+      <c r="Q61" s="14"/>
+      <c r="R61" s="14"/>
+      <c r="S61" s="14"/>
+      <c r="T61" s="17" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="U61" s="14"/>
+      <c r="V61" s="44" t="n">
+        <f aca="false">SUM(N61:U61)</f>
         <v>-64406</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="B61" s="51" t="n">
-        <f aca="false">SUM(B50:B60)</f>
-        <v>0</v>
-      </c>
-      <c r="C61" s="22" t="n">
-        <f aca="false">SUM(C50:C60)</f>
+    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="51" t="n">
+        <f aca="false">SUM(B51:B61)</f>
+        <v>0</v>
+      </c>
+      <c r="C62" s="22" t="n">
+        <f aca="false">SUM(C51:C61)</f>
         <v>80000</v>
       </c>
-      <c r="D61" s="21" t="n">
-        <f aca="false">SUM(D50:D60)</f>
+      <c r="D62" s="21" t="n">
+        <f aca="false">SUM(D51:D61)</f>
         <v>50000</v>
       </c>
-      <c r="E61" s="21" t="n">
-        <f aca="false">SUM(E50:E60)</f>
+      <c r="E62" s="21" t="n">
+        <f aca="false">SUM(E51:E61)</f>
         <v>-22200</v>
       </c>
-      <c r="F61" s="21" t="n">
-        <f aca="false">SUM(F50:F60)</f>
+      <c r="F62" s="21" t="n">
+        <f aca="false">SUM(F51:F61)</f>
         <v>-100000</v>
       </c>
-      <c r="G61" s="21" t="n">
-        <f aca="false">SUM(G50:G60)</f>
+      <c r="G62" s="21" t="n">
+        <f aca="false">SUM(G51:G61)</f>
         <v>-1200</v>
       </c>
-      <c r="H61" s="21" t="n">
-        <f aca="false">SUM(H50:H60)</f>
+      <c r="H62" s="21" t="n">
+        <f aca="false">SUM(H51:H61)</f>
         <v>122000</v>
       </c>
-      <c r="I61" s="21" t="n">
-        <f aca="false">SUM(I50:I60)</f>
+      <c r="I62" s="21" t="n">
+        <f aca="false">SUM(I51:I61)</f>
         <v>-1000</v>
       </c>
-      <c r="J61" s="21" t="n">
-        <f aca="false">SUM(J50:J60)</f>
-        <v>0</v>
-      </c>
-      <c r="K61" s="21" t="n">
-        <f aca="false">SUM(K50:K60)</f>
-        <v>0</v>
-      </c>
-      <c r="L61" s="21" t="n">
-        <f aca="false">SUM(L50:L60)</f>
-        <v>0</v>
-      </c>
-      <c r="M61" s="52" t="n">
-        <f aca="false">SUM(M50:M60)</f>
+      <c r="J62" s="21" t="n">
+        <f aca="false">SUM(J51:J61)</f>
+        <v>0</v>
+      </c>
+      <c r="K62" s="21" t="n">
+        <f aca="false">SUM(K51:K61)</f>
+        <v>0</v>
+      </c>
+      <c r="L62" s="21" t="n">
+        <f aca="false">SUM(L51:L61)</f>
+        <v>0</v>
+      </c>
+      <c r="M62" s="52" t="n">
+        <f aca="false">SUM(M51:M61)</f>
         <v>127600</v>
       </c>
-      <c r="N61" s="21" t="n">
-        <f aca="false">SUM(N50:N60)</f>
+      <c r="N62" s="21" t="n">
+        <f aca="false">SUM(N51:N61)</f>
         <v>34594</v>
       </c>
-      <c r="O61" s="21" t="n">
-        <f aca="false">SUM(O50:O60)</f>
+      <c r="O62" s="21" t="n">
+        <f aca="false">SUM(O51:O61)</f>
         <v>-155000</v>
       </c>
-      <c r="P61" s="21" t="n">
-        <f aca="false">SUM(P50:P60)</f>
+      <c r="P62" s="21" t="n">
+        <f aca="false">SUM(P51:P61)</f>
         <v>156000</v>
       </c>
-      <c r="Q61" s="21" t="n">
-        <f aca="false">SUM(Q50:Q60)</f>
+      <c r="Q62" s="21" t="n">
+        <f aca="false">SUM(Q51:Q61)</f>
         <v>250</v>
       </c>
-      <c r="R61" s="21" t="n">
-        <f aca="false">SUM(R50:R60)</f>
+      <c r="R62" s="21" t="n">
+        <f aca="false">SUM(R51:R61)</f>
         <v>-1000</v>
       </c>
-      <c r="S61" s="21" t="n">
-        <f aca="false">SUM(S50:S60)</f>
-        <v>0</v>
-      </c>
-      <c r="T61" s="21" t="n">
-        <f aca="false">SUM(T50:T60)</f>
+      <c r="S62" s="21" t="n">
+        <f aca="false">SUM(S51:S61)</f>
+        <v>0</v>
+      </c>
+      <c r="T62" s="21" t="n">
+        <f aca="false">SUM(T51:T61)</f>
         <v>-51000</v>
       </c>
-      <c r="U61" s="21" t="n">
-        <f aca="false">SUM(U50:U60)</f>
+      <c r="U62" s="21" t="n">
+        <f aca="false">SUM(U51:U61)</f>
         <v>-15435</v>
       </c>
-      <c r="V61" s="52" t="n">
-        <f aca="false">SUM(V50:V60)</f>
+      <c r="V62" s="52" t="n">
+        <f aca="false">SUM(V51:V61)</f>
         <v>-31591</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="B62" s="24"/>
-      <c r="C62" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="24" t="n">
-        <f aca="false">C63</f>
-        <v>80000</v>
-      </c>
-      <c r="E62" s="24" t="n">
-        <f aca="false">D63</f>
-        <v>130000</v>
-      </c>
-      <c r="F62" s="24" t="n">
-        <f aca="false">E63</f>
-        <v>107800</v>
-      </c>
-      <c r="G62" s="24" t="n">
-        <f aca="false">F63</f>
-        <v>7800</v>
-      </c>
-      <c r="H62" s="24" t="n">
-        <f aca="false">G63</f>
-        <v>6600</v>
-      </c>
-      <c r="I62" s="24" t="n">
-        <f aca="false">H63</f>
-        <v>128600</v>
-      </c>
-      <c r="J62" s="24" t="n">
-        <f aca="false">I63</f>
-        <v>127600</v>
-      </c>
-      <c r="K62" s="24" t="n">
-        <f aca="false">J63</f>
-        <v>127600</v>
-      </c>
-      <c r="L62" s="24" t="n">
-        <f aca="false">K63</f>
-        <v>127600</v>
-      </c>
-      <c r="M62" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N62" s="24" t="n">
-        <f aca="false">M63</f>
-        <v>127600</v>
-      </c>
-      <c r="O62" s="24" t="n">
-        <f aca="false">N63</f>
-        <v>162194</v>
-      </c>
-      <c r="P62" s="24" t="n">
-        <f aca="false">O63</f>
-        <v>7194</v>
-      </c>
-      <c r="Q62" s="24" t="n">
-        <f aca="false">P63</f>
-        <v>163194</v>
-      </c>
-      <c r="R62" s="24" t="n">
-        <f aca="false">Q63</f>
-        <v>163444</v>
-      </c>
-      <c r="S62" s="24" t="n">
-        <f aca="false">R63</f>
-        <v>162444</v>
-      </c>
-      <c r="T62" s="24" t="n">
-        <f aca="false">S63</f>
-        <v>162444</v>
-      </c>
-      <c r="U62" s="24" t="n">
-        <f aca="false">T63</f>
-        <v>111444</v>
-      </c>
-      <c r="V62" s="24" t="n">
-        <f aca="false">M63</f>
-        <v>127600</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="B63" s="22"/>
-      <c r="C63" s="22" t="n">
-        <f aca="false">C62+C61</f>
+      <c r="B63" s="24"/>
+      <c r="C63" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="24" t="n">
+        <f aca="false">C64</f>
         <v>80000</v>
       </c>
-      <c r="D63" s="22" t="n">
-        <f aca="false">D62+D61</f>
+      <c r="E63" s="24" t="n">
+        <f aca="false">D64</f>
         <v>130000</v>
       </c>
-      <c r="E63" s="22" t="n">
-        <f aca="false">E62+E61</f>
+      <c r="F63" s="24" t="n">
+        <f aca="false">E64</f>
         <v>107800</v>
       </c>
-      <c r="F63" s="22" t="n">
-        <f aca="false">F62+F61</f>
+      <c r="G63" s="24" t="n">
+        <f aca="false">F64</f>
         <v>7800</v>
       </c>
-      <c r="G63" s="22" t="n">
-        <f aca="false">G62+G61</f>
+      <c r="H63" s="24" t="n">
+        <f aca="false">G64</f>
         <v>6600</v>
       </c>
-      <c r="H63" s="22" t="n">
-        <f aca="false">H62+H61</f>
+      <c r="I63" s="24" t="n">
+        <f aca="false">H64</f>
         <v>128600</v>
       </c>
-      <c r="I63" s="22" t="n">
-        <f aca="false">I62+I61</f>
+      <c r="J63" s="24" t="n">
+        <f aca="false">I64</f>
         <v>127600</v>
       </c>
-      <c r="J63" s="22" t="n">
-        <f aca="false">J62+J61</f>
+      <c r="K63" s="24" t="n">
+        <f aca="false">J64</f>
         <v>127600</v>
       </c>
-      <c r="K63" s="22" t="n">
-        <f aca="false">K62+K61</f>
+      <c r="L63" s="24" t="n">
+        <f aca="false">K64</f>
         <v>127600</v>
       </c>
-      <c r="L63" s="22" t="n">
-        <f aca="false">L62+L61</f>
+      <c r="M63" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" s="24" t="n">
+        <f aca="false">M64</f>
         <v>127600</v>
       </c>
-      <c r="M63" s="22" t="n">
-        <f aca="false">M62+M61</f>
+      <c r="O63" s="24" t="n">
+        <f aca="false">N64</f>
+        <v>162194</v>
+      </c>
+      <c r="P63" s="24" t="n">
+        <f aca="false">O64</f>
+        <v>7194</v>
+      </c>
+      <c r="Q63" s="24" t="n">
+        <f aca="false">P64</f>
+        <v>163194</v>
+      </c>
+      <c r="R63" s="24" t="n">
+        <f aca="false">Q64</f>
+        <v>163444</v>
+      </c>
+      <c r="S63" s="24" t="n">
+        <f aca="false">R64</f>
+        <v>162444</v>
+      </c>
+      <c r="T63" s="24" t="n">
+        <f aca="false">S64</f>
+        <v>162444</v>
+      </c>
+      <c r="U63" s="24" t="n">
+        <f aca="false">T64</f>
+        <v>111444</v>
+      </c>
+      <c r="V63" s="24" t="n">
+        <f aca="false">M64</f>
         <v>127600</v>
       </c>
-      <c r="N63" s="22" t="n">
-        <f aca="false">N62+N61</f>
+    </row>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="B64" s="22"/>
+      <c r="C64" s="22" t="n">
+        <f aca="false">C63+C62</f>
+        <v>80000</v>
+      </c>
+      <c r="D64" s="22" t="n">
+        <f aca="false">D63+D62</f>
+        <v>130000</v>
+      </c>
+      <c r="E64" s="22" t="n">
+        <f aca="false">E63+E62</f>
+        <v>107800</v>
+      </c>
+      <c r="F64" s="22" t="n">
+        <f aca="false">F63+F62</f>
+        <v>7800</v>
+      </c>
+      <c r="G64" s="22" t="n">
+        <f aca="false">G63+G62</f>
+        <v>6600</v>
+      </c>
+      <c r="H64" s="22" t="n">
+        <f aca="false">H63+H62</f>
+        <v>128600</v>
+      </c>
+      <c r="I64" s="22" t="n">
+        <f aca="false">I63+I62</f>
+        <v>127600</v>
+      </c>
+      <c r="J64" s="22" t="n">
+        <f aca="false">J63+J62</f>
+        <v>127600</v>
+      </c>
+      <c r="K64" s="22" t="n">
+        <f aca="false">K63+K62</f>
+        <v>127600</v>
+      </c>
+      <c r="L64" s="22" t="n">
+        <f aca="false">L63+L62</f>
+        <v>127600</v>
+      </c>
+      <c r="M64" s="22" t="n">
+        <f aca="false">M63+M62</f>
+        <v>127600</v>
+      </c>
+      <c r="N64" s="22" t="n">
+        <f aca="false">N63+N62</f>
         <v>162194</v>
       </c>
-      <c r="O63" s="22" t="n">
-        <f aca="false">O62+O61</f>
+      <c r="O64" s="22" t="n">
+        <f aca="false">O63+O62</f>
         <v>7194</v>
       </c>
-      <c r="P63" s="22" t="n">
-        <f aca="false">P62+P61</f>
+      <c r="P64" s="22" t="n">
+        <f aca="false">P63+P62</f>
         <v>163194</v>
       </c>
-      <c r="Q63" s="22" t="n">
-        <f aca="false">Q62+Q61</f>
+      <c r="Q64" s="22" t="n">
+        <f aca="false">Q63+Q62</f>
         <v>163444</v>
       </c>
-      <c r="R63" s="22" t="n">
-        <f aca="false">R62+R61</f>
+      <c r="R64" s="22" t="n">
+        <f aca="false">R63+R62</f>
         <v>162444</v>
       </c>
-      <c r="S63" s="22" t="n">
-        <f aca="false">S62+S61</f>
+      <c r="S64" s="22" t="n">
+        <f aca="false">S63+S62</f>
         <v>162444</v>
       </c>
-      <c r="T63" s="22" t="n">
-        <f aca="false">T62+T61</f>
+      <c r="T64" s="22" t="n">
+        <f aca="false">T63+T62</f>
         <v>111444</v>
       </c>
-      <c r="U63" s="22" t="n">
-        <f aca="false">U62+U61</f>
+      <c r="U64" s="22" t="n">
+        <f aca="false">U63+U62</f>
         <v>96009</v>
       </c>
-      <c r="V63" s="22" t="n">
-        <f aca="false">V62+V61</f>
+      <c r="V64" s="22" t="n">
+        <f aca="false">V63+V62</f>
         <v>96009</v>
       </c>
     </row>

</xml_diff>